<commit_message>
Remove temporary Excel file
</commit_message>
<xml_diff>
--- a/Campus_Placement_Intelligence_Final.xlsx
+++ b/Campus_Placement_Intelligence_Final.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7500" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7500" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Analysis" sheetId="5" r:id="rId1"/>
@@ -8901,15 +8901,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:colOff>19051</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>4391025</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
+      <xdr:colOff>3352800</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8931,15 +8931,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>4471987</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:colOff>3405187</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>390525</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>